<commit_message>
feat<product>: fix Excel import bugs - fix date added, qty, images, specs and color fields
</commit_message>
<xml_diff>
--- a/test_data/product_import_template_FINAL.xlsx
+++ b/test_data/product_import_template_FINAL.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QAC\OneDrive - ptit.edu.vn\Desktop\EyseGlass\E-commerce-platform-for-Eyewear-retail\test_data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E33454B-9397-4FF8-B7B4-57B94A4F9F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -29,15 +23,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="94">
   <si>
     <t>Name</t>
   </si>
@@ -186,6 +177,18 @@
     <t>#1A1A1A</t>
   </si>
   <si>
+    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854784/eyewear_import/MV2001N-5S_img3.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854784/eyewear_import/MV2001N-5S_img2.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854783/eyewear_import/MV2001N-5S_img1.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854782/eyewear_import/MV2001N-5S_img0.webp</t>
+  </si>
+  <si>
     <t>Gong Kinh RayBan Classic</t>
   </si>
   <si>
@@ -234,6 +237,12 @@
     <t>#C5A028</t>
   </si>
   <si>
+    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773850666/glasses-store/products/file_ye9756.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773850663/glasses-store/products/file_coh2ea.png</t>
+  </si>
+  <si>
     <t>HUONG DAN CHEN ANH (5 anh cho moi san pham)</t>
   </si>
   <si>
@@ -301,84 +310,201 @@
   </si>
   <si>
     <t>SKU la bat buoc va phai khac nhau. SKU da ton tai =&gt; cap nhat san pham.</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773850666/glasses-store/products/file_ye9756.png</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773850663/glasses-store/products/file_coh2ea.png</t>
-  </si>
-  <si>
-    <t>sayhi</t>
-  </si>
-  <si>
-    <t>RB-001-GLC</t>
-  </si>
-  <si>
-    <t>RB-001-GLE</t>
-  </si>
-  <si>
-    <t>saybye</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854795/eyewear_import/SR1010X-5A_img0.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854794/eyewear_import/OR1060X-5S_img4.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854784/eyewear_import/MV2001N-5S_img3.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854784/eyewear_import/MV2001N-5S_img2.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854783/eyewear_import/MV2001N-5S_img1.webp</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854782/eyewear_import/MV2001N-5S_img0.webp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF1F4E79"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC55A11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color rgb="FF1F4E79"/>
-      <name val="Calibri"/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFC55A11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -387,31 +513,222 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC55A11"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF3FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC55A11"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEBF3FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -419,44 +736,327 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -741,14 +1341,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:AF3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -776,576 +1376,403 @@
     <col min="29" max="32" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="32.1" customHeight="1" spans="1:32">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AD1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AE1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AF1" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" ht="80.1" customHeight="1" spans="1:32">
+      <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="5">
         <v>2500000</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="5">
         <v>2100000</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="V2" s="4">
+      <c r="V2" s="5">
         <v>0</v>
       </c>
-      <c r="W2" s="4">
+      <c r="W2" s="5">
         <v>25</v>
       </c>
-      <c r="X2" s="4">
+      <c r="X2" s="5">
         <v>54</v>
       </c>
-      <c r="Y2" s="4">
+      <c r="Y2" s="5">
         <v>18</v>
       </c>
-      <c r="Z2" s="4">
+      <c r="Z2" s="5">
         <v>145</v>
       </c>
-      <c r="AA2" s="4">
+      <c r="AA2" s="5">
         <v>28</v>
       </c>
       <c r="AB2" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="AC2" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="AD2" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="AF2" s="8" t="s">
-        <v>99</v>
+        <v>49</v>
+      </c>
+      <c r="AC2" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD2" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF2" s="9" t="s">
+        <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:32" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="5" t="s">
+    <row r="3" ht="80.1" customHeight="1" spans="1:29">
+      <c r="A3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="6">
+        <v>1200000</v>
+      </c>
+      <c r="H3" s="6">
+        <v>980000</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="V3" s="6">
+        <v>0</v>
+      </c>
+      <c r="W3" s="6">
+        <v>30</v>
+      </c>
+      <c r="X3" s="6">
         <v>52</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" s="5">
-        <v>1200000</v>
-      </c>
-      <c r="H3" s="5">
-        <v>980000</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="V3" s="5">
-        <v>0</v>
-      </c>
-      <c r="W3" s="5">
-        <v>30</v>
-      </c>
-      <c r="X3" s="5">
-        <v>52</v>
-      </c>
-      <c r="Y3" s="5">
+      <c r="Y3" s="6">
         <v>17</v>
       </c>
-      <c r="Z3" s="5">
+      <c r="Z3" s="6">
         <v>140</v>
       </c>
-      <c r="AA3" s="5">
+      <c r="AA3" s="6">
         <v>22</v>
       </c>
-      <c r="AB3" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="AC3" s="8" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="5">
-        <v>1200000</v>
-      </c>
-      <c r="H4" s="5">
-        <v>980000</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="T4" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="U4" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="V4" s="5">
-        <v>0</v>
-      </c>
-      <c r="W4" s="5">
-        <v>30</v>
-      </c>
-      <c r="X4" s="5">
-        <v>52</v>
-      </c>
-      <c r="Y4" s="5">
-        <v>17</v>
-      </c>
-      <c r="Z4" s="5">
-        <v>140</v>
-      </c>
-      <c r="AA4" s="5">
-        <v>22</v>
-      </c>
-      <c r="AB4" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="AC4" s="8" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="5">
-        <v>1200000</v>
-      </c>
-      <c r="H5" s="5">
-        <v>980000</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="R5" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S5" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="T5" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="U5" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="V5" s="5">
-        <v>0</v>
-      </c>
-      <c r="W5" s="5">
-        <v>30</v>
-      </c>
-      <c r="X5" s="5">
-        <v>52</v>
-      </c>
-      <c r="Y5" s="5">
-        <v>17</v>
-      </c>
-      <c r="Z5" s="5">
-        <v>140</v>
-      </c>
-      <c r="AA5" s="5">
-        <v>22</v>
-      </c>
-      <c r="AB5" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC5" s="8" t="s">
-        <v>95</v>
+      <c r="AB3" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC3" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="AB2" r:id="rId1" xr:uid="{1EA07686-1978-41C5-B0E5-6B08A6F152A1}"/>
-    <hyperlink ref="AC2" r:id="rId2" xr:uid="{9E6FBC63-941A-4934-B29E-F8023BDC13CF}"/>
-    <hyperlink ref="AB3" r:id="rId3" xr:uid="{D074B2E4-F980-4C54-B485-99B5681B1EBC}"/>
-    <hyperlink ref="AC3" r:id="rId4" xr:uid="{BD593F5B-B665-482F-B247-025FFA73C8E4}"/>
-    <hyperlink ref="AB4" r:id="rId5" xr:uid="{7958F751-77EC-4447-9956-DC242AF8E98E}"/>
-    <hyperlink ref="AC4" r:id="rId6" xr:uid="{1D552509-2436-4D5B-92A8-9C1565686593}"/>
-    <hyperlink ref="AB5" r:id="rId7" xr:uid="{680FDB71-0F80-4277-8710-DA48D2EA0B29}"/>
-    <hyperlink ref="AC5" r:id="rId8" xr:uid="{18D26A82-58EA-4723-B608-71457DDD8641}"/>
-    <hyperlink ref="AD2" r:id="rId9" xr:uid="{7B4D85AF-01F1-4D6C-94C3-9FF4B01A8722}"/>
-    <hyperlink ref="AF2" r:id="rId10" xr:uid="{7F1A45CD-DE2D-4C64-A054-E68649A14257}"/>
+    <hyperlink ref="AB2" r:id="rId1" display="https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854784/eyewear_import/MV2001N-5S_img3.webp"/>
+    <hyperlink ref="AC2" r:id="rId2" display="https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854784/eyewear_import/MV2001N-5S_img2.webp"/>
+    <hyperlink ref="AB3" r:id="rId3" display="https://res.cloudinary.com/dfk16iu6d/image/upload/v1773850666/glasses-store/products/file_ye9756.png"/>
+    <hyperlink ref="AC3" r:id="rId4" display="https://res.cloudinary.com/dfk16iu6d/image/upload/v1773850663/glasses-store/products/file_coh2ea.png"/>
+    <hyperlink ref="AD2" r:id="rId5" display="https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854783/eyewear_import/MV2001N-5S_img1.webp"/>
+    <hyperlink ref="AF2" r:id="rId6" display="https://res.cloudinary.com/dfk16iu6d/image/upload/v1773854782/eyewear_import/MV2001N-5S_img0.webp"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>65</v>
+    <row r="1" ht="18.75" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>66</v>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>68</v>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>70</v>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>72</v>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>74</v>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>76</v>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>78</v>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>80</v>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>82</v>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>84</v>
+    <row r="12" spans="1:2">
+      <c r="A12" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>86</v>
+    <row r="13" spans="1:2">
+      <c r="A13" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>